<commit_message>
Update dashboard logic, titles, and root files
</commit_message>
<xml_diff>
--- a/collocation_tracking_pm25.xlsx
+++ b/collocation_tracking_pm25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nlambini\Desktop\Collocation Tracking Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81C61C1A-2EF6-4BCF-BB6D-5E31B7270B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E806514-21CD-4003-8998-02CF79DA6963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B5225731-ACF7-4F9B-B48D-4E756CF11B97}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="83">
   <si>
     <t>Method Type</t>
   </si>
@@ -90,9 +90,6 @@
   </si>
   <si>
     <t>Corcoran - Patterson (SJV)</t>
-  </si>
-  <si>
-    <t>Del Paso Manor (Sac Metro)</t>
   </si>
   <si>
     <t>El Rio (Ventura)</t>
@@ -658,7 +655,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24C0B712-3E18-423F-B8D0-5A08FB824E46}">
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.90625" bestFit="1" customWidth="1"/>
@@ -690,10 +687,10 @@
         <v>209</v>
       </c>
       <c r="B2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" t="s">
         <v>63</v>
-      </c>
-      <c r="C2" t="s">
-        <v>64</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -707,10 +704,10 @@
         <v>209</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
@@ -721,10 +718,10 @@
         <v>209</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D4" t="s">
         <v>7</v>
@@ -735,10 +732,10 @@
         <v>209</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -749,10 +746,10 @@
         <v>209</v>
       </c>
       <c r="B6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
@@ -763,10 +760,10 @@
         <v>209</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D7" t="s">
         <v>7</v>
@@ -777,10 +774,10 @@
         <v>209</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D8" t="s">
         <v>7</v>
@@ -791,10 +788,10 @@
         <v>209</v>
       </c>
       <c r="B9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D9" t="s">
         <v>7</v>
@@ -805,10 +802,10 @@
         <v>143</v>
       </c>
       <c r="B10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" t="s">
         <v>72</v>
-      </c>
-      <c r="C10" t="s">
-        <v>73</v>
       </c>
       <c r="D10" t="s">
         <v>7</v>
@@ -822,10 +819,10 @@
         <v>143</v>
       </c>
       <c r="B11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D11" t="s">
         <v>7</v>
@@ -836,10 +833,10 @@
         <v>145</v>
       </c>
       <c r="B12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" t="s">
         <v>75</v>
-      </c>
-      <c r="C12" t="s">
-        <v>76</v>
       </c>
       <c r="D12" t="s">
         <v>7</v>
@@ -853,10 +850,10 @@
         <v>145</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D13" t="s">
         <v>7</v>
@@ -867,10 +864,10 @@
         <v>145</v>
       </c>
       <c r="B14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D14" t="s">
         <v>7</v>
@@ -881,10 +878,10 @@
         <v>181</v>
       </c>
       <c r="B15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C15" t="s">
         <v>79</v>
-      </c>
-      <c r="C15" t="s">
-        <v>80</v>
       </c>
       <c r="D15" t="s">
         <v>7</v>
@@ -898,10 +895,10 @@
         <v>638</v>
       </c>
       <c r="B16" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" t="s">
         <v>81</v>
-      </c>
-      <c r="C16" t="s">
-        <v>82</v>
       </c>
       <c r="D16" t="s">
         <v>7</v>
@@ -915,10 +912,10 @@
         <v>638</v>
       </c>
       <c r="B17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D17" t="s">
         <v>7</v>
@@ -1108,6 +1105,9 @@
       <c r="D30" t="s">
         <v>7</v>
       </c>
+      <c r="E30" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31">
@@ -1122,9 +1122,6 @@
       <c r="D31" t="s">
         <v>7</v>
       </c>
-      <c r="E31" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32">
@@ -1139,8 +1136,11 @@
       <c r="D32" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E32" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>170</v>
       </c>
@@ -1153,11 +1153,8 @@
       <c r="D33" t="s">
         <v>7</v>
       </c>
-      <c r="E33" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>170</v>
       </c>
@@ -1171,7 +1168,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>170</v>
       </c>
@@ -1185,7 +1182,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>170</v>
       </c>
@@ -1199,7 +1196,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>170</v>
       </c>
@@ -1213,7 +1210,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>170</v>
       </c>
@@ -1227,7 +1224,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>170</v>
       </c>
@@ -1241,7 +1238,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>170</v>
       </c>
@@ -1255,7 +1252,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>170</v>
       </c>
@@ -1269,7 +1266,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>170</v>
       </c>
@@ -1283,7 +1280,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>170</v>
       </c>
@@ -1297,7 +1294,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>170</v>
       </c>
@@ -1311,7 +1308,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>170</v>
       </c>
@@ -1325,7 +1322,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>170</v>
       </c>
@@ -1339,7 +1336,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>170</v>
       </c>
@@ -1353,7 +1350,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>170</v>
       </c>
@@ -1408,6 +1405,9 @@
       <c r="D51" t="s">
         <v>7</v>
       </c>
+      <c r="E51" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52">
@@ -1439,9 +1439,6 @@
       <c r="D53" t="s">
         <v>7</v>
       </c>
-      <c r="E53" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54">
@@ -1526,6 +1523,9 @@
       <c r="D59" t="s">
         <v>7</v>
       </c>
+      <c r="E59" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60">
@@ -1540,9 +1540,6 @@
       <c r="D60" t="s">
         <v>7</v>
       </c>
-      <c r="E60" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61">
@@ -1641,6 +1638,9 @@
       <c r="D67" t="s">
         <v>7</v>
       </c>
+      <c r="E67" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68">
@@ -1655,9 +1655,6 @@
       <c r="D68" t="s">
         <v>7</v>
       </c>
-      <c r="E68" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69">
@@ -1714,21 +1711,7 @@
       <c r="D72" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A73">
-        <v>170</v>
-      </c>
-      <c r="B73" t="s">
-        <v>5</v>
-      </c>
-      <c r="C73" t="s">
-        <v>62</v>
-      </c>
-      <c r="D73" t="s">
-        <v>7</v>
-      </c>
-      <c r="E73" t="s">
+      <c r="E72" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>